<commit_message>
MIT license, descriptive README, dates as labels in the examples
Assessment dates may be labels such as 'Date 1' (files: date_1); the examples use Date 1 and Date 2. README: new title and introduction, Example 1 shown in four rows (design, assessed plots, score maps, distribution).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/data/example_1_merged_plots.xlsx
+++ b/examples/data/example_1_merged_plots.xlsx
@@ -8,8 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="field_map" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="20250815" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="20250905" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="date_1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="date_2" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Figures of one layout share size and plot shapes; justified README
Design, coverage and map figures use a fixed frame (title band, map at a fixed scale, legend band); the distribution chart takes the same width. Example 1: wider plots, and Date 2 re-assesses every Date 1 plot plus new ones. README text justified.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/data/example_1_merged_plots.xlsx
+++ b/examples/data/example_1_merged_plots.xlsx
@@ -1434,7 +1434,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -1444,7 +1444,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1452,7 +1452,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1462,7 +1462,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1470,7 +1470,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -1480,7 +1480,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1488,7 +1488,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1506,7 +1506,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1516,7 +1516,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1524,7 +1524,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1534,7 +1534,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -1542,7 +1542,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1552,7 +1552,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1570,7 +1570,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1578,7 +1578,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1588,7 +1588,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1596,7 +1596,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1614,7 +1614,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1642,7 +1642,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1650,7 +1650,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1660,7 +1660,7 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1668,7 +1668,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1678,7 +1678,7 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1696,7 +1696,7 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1704,7 +1704,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1714,7 +1714,7 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1722,7 +1722,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1740,7 +1740,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1750,7 +1750,7 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1758,7 +1758,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1768,7 +1768,7 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1776,7 +1776,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1786,7 +1786,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -1794,7 +1794,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1804,7 +1804,7 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1822,15 +1822,15 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>157</v>
+        <v>203</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>BLOCK A</t>
+          <t>BLOCK B</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1840,7 +1840,7 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -1848,7 +1848,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1858,7 +1858,7 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -1866,7 +1866,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1876,7 +1876,7 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -1884,7 +1884,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -1894,7 +1894,7 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -1902,7 +1902,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -1912,7 +1912,7 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -1920,7 +1920,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -1930,7 +1930,7 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -1956,7 +1956,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1966,7 +1966,7 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -1974,7 +1974,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1984,7 +1984,7 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -1992,7 +1992,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -2002,7 +2002,7 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2010,7 +2010,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -2020,7 +2020,7 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2028,7 +2028,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2038,7 +2038,7 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -2046,7 +2046,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -2056,7 +2056,7 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -2074,7 +2074,7 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -2082,7 +2082,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -2092,7 +2092,7 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -2100,7 +2100,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -2110,7 +2110,7 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -2118,7 +2118,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -2128,7 +2128,7 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -2136,7 +2136,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -2146,7 +2146,7 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -2154,7 +2154,7 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -2164,7 +2164,7 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -2172,7 +2172,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -2182,7 +2182,7 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -2200,7 +2200,7 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>248</v>
+        <v>254</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -2208,7 +2208,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -2218,7 +2218,7 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -2226,7 +2226,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -2236,7 +2236,7 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -2244,7 +2244,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -2254,7 +2254,7 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -2262,7 +2262,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -2272,7 +2272,7 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -2280,7 +2280,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -2290,15 +2290,15 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>256</v>
+        <v>310</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>BLOCK B</t>
+          <t>BLOCK C</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -2308,15 +2308,15 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>258</v>
+        <v>317</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>BLOCK B</t>
+          <t>BLOCK C</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -2326,7 +2326,7 @@
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>302</v>
+        <v>318</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -2334,7 +2334,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -2344,7 +2344,7 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>308</v>
+        <v>319</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -2352,7 +2352,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -2362,7 +2362,7 @@
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>309</v>
+        <v>320</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -2370,7 +2370,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -2380,7 +2380,7 @@
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>312</v>
+        <v>322</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -2388,7 +2388,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>52</v>
+        <v>15</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>313</v>
+        <v>324</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -2406,7 +2406,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>43</v>
+        <v>25</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -2416,7 +2416,7 @@
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>316</v>
+        <v>325</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
@@ -2424,7 +2424,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -2434,7 +2434,7 @@
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>318</v>
+        <v>326</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -2452,7 +2452,7 @@
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>320</v>
+        <v>329</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
@@ -2460,7 +2460,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -2470,7 +2470,7 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>321</v>
+        <v>330</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
@@ -2478,7 +2478,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>21</v>
+        <v>56</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -2488,7 +2488,7 @@
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>324</v>
+        <v>331</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
@@ -2496,7 +2496,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -2506,7 +2506,7 @@
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
@@ -2514,7 +2514,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -2524,7 +2524,7 @@
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -2532,7 +2532,7 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -2542,7 +2542,7 @@
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>327</v>
+        <v>335</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
@@ -2550,7 +2550,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -2560,7 +2560,7 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -2578,15 +2578,15 @@
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>333</v>
+        <v>405</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>BLOCK C</t>
+          <t>BLOCK D</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -2596,15 +2596,15 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>335</v>
+        <v>407</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>BLOCK C</t>
+          <t>BLOCK D</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -2614,15 +2614,15 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>336</v>
+        <v>409</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>BLOCK C</t>
+          <t>BLOCK D</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -2632,15 +2632,15 @@
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>340</v>
+        <v>412</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>BLOCK C</t>
+          <t>BLOCK D</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -2650,7 +2650,7 @@
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>404</v>
+        <v>415</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
@@ -2658,7 +2658,7 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -2668,7 +2668,7 @@
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>405</v>
+        <v>418</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -2676,7 +2676,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -2686,7 +2686,7 @@
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>408</v>
+        <v>419</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -2704,7 +2704,7 @@
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>410</v>
+        <v>421</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
@@ -2712,7 +2712,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>411</v>
+        <v>424</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
@@ -2730,7 +2730,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -2740,7 +2740,7 @@
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>412</v>
+        <v>427</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -2758,7 +2758,7 @@
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>413</v>
+        <v>428</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
@@ -2766,7 +2766,7 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -2776,7 +2776,7 @@
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>420</v>
+        <v>430</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
@@ -2784,7 +2784,7 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>57</v>
+        <v>16</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -2794,7 +2794,7 @@
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>421</v>
+        <v>432</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
@@ -2802,7 +2802,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>46</v>
+        <v>17</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -2812,7 +2812,7 @@
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>422</v>
+        <v>436</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -2830,7 +2830,7 @@
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>429</v>
+        <v>437</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
@@ -2838,7 +2838,7 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -2848,7 +2848,7 @@
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>432</v>
+        <v>438</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
@@ -2856,7 +2856,7 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -2866,7 +2866,7 @@
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>435</v>
+        <v>440</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -2874,7 +2874,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -2884,7 +2884,7 @@
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>441</v>
+        <v>446</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
@@ -2892,7 +2892,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -2902,7 +2902,7 @@
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>443</v>
+        <v>447</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
@@ -2910,7 +2910,7 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -2920,7 +2920,7 @@
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
@@ -2928,7 +2928,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -2947,7 +2947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D127"/>
+  <dimension ref="A1:D148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2974,7 +2974,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -2982,7 +2982,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2992,7 +2992,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -3000,7 +3000,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -3010,7 +3010,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -3018,7 +3018,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -3028,7 +3028,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -3036,7 +3036,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -3046,7 +3046,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -3054,7 +3054,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -3064,7 +3064,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -3082,7 +3082,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -3090,7 +3090,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -3100,7 +3100,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -3108,7 +3108,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -3118,7 +3118,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -3126,7 +3126,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -3136,7 +3136,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -3144,7 +3144,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -3154,7 +3154,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -3162,7 +3162,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -3172,7 +3172,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -3180,7 +3180,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -3190,7 +3190,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -3216,7 +3216,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -3226,7 +3226,7 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -3234,7 +3234,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -3244,7 +3244,7 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -3252,7 +3252,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -3262,7 +3262,7 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -3280,7 +3280,7 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -3288,7 +3288,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>52</v>
+        <v>66</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -3298,7 +3298,7 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -3306,7 +3306,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -3316,7 +3316,7 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -3334,7 +3334,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -3342,7 +3342,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -3352,7 +3352,7 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -3360,7 +3360,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -3370,7 +3370,7 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -3378,7 +3378,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -3388,7 +3388,7 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -3396,7 +3396,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -3406,7 +3406,7 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -3414,7 +3414,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -3424,7 +3424,7 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -3432,7 +3432,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -3442,7 +3442,7 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -3450,7 +3450,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -3460,7 +3460,7 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -3468,7 +3468,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -3478,7 +3478,7 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -3486,7 +3486,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -3496,7 +3496,7 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -3504,7 +3504,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -3514,7 +3514,7 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -3522,7 +3522,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -3532,7 +3532,7 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -3540,7 +3540,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -3550,7 +3550,7 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -3568,7 +3568,7 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -3586,7 +3586,7 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3594,7 +3594,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -3604,7 +3604,7 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3612,7 +3612,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -3622,7 +3622,7 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -3666,7 +3666,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -3684,7 +3684,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -3702,7 +3702,7 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -3720,7 +3720,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -3738,7 +3738,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -3756,7 +3756,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -3766,7 +3766,7 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -3774,7 +3774,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -3784,7 +3784,7 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -3792,7 +3792,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -3802,7 +3802,7 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -3810,7 +3810,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -3820,7 +3820,7 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -3828,7 +3828,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -3838,7 +3838,7 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -3846,7 +3846,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -3856,7 +3856,7 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -3864,7 +3864,7 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -3874,7 +3874,7 @@
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -3882,7 +3882,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -3892,7 +3892,7 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -3900,7 +3900,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -3918,7 +3918,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -3928,7 +3928,7 @@
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -3936,7 +3936,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>81</v>
+        <v>59</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -3946,7 +3946,7 @@
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -3954,7 +3954,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -3964,7 +3964,7 @@
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
@@ -3972,7 +3972,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -4000,7 +4000,7 @@
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
@@ -4008,7 +4008,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -4018,7 +4018,7 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
@@ -4026,7 +4026,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -4036,7 +4036,7 @@
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
@@ -4044,7 +4044,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -4054,7 +4054,7 @@
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
@@ -4062,7 +4062,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -4072,7 +4072,7 @@
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -4080,7 +4080,7 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -4090,7 +4090,7 @@
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
@@ -4098,7 +4098,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -4108,7 +4108,7 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
@@ -4116,7 +4116,7 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -4126,7 +4126,7 @@
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -4134,7 +4134,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -4144,7 +4144,7 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
@@ -4152,7 +4152,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -4162,7 +4162,7 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
@@ -4170,7 +4170,7 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -4180,7 +4180,7 @@
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
@@ -4188,7 +4188,7 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -4198,7 +4198,7 @@
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
@@ -4206,7 +4206,7 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -4216,7 +4216,7 @@
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -4224,7 +4224,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -4234,7 +4234,7 @@
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
@@ -4242,7 +4242,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -4252,7 +4252,7 @@
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
@@ -4260,7 +4260,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -4270,7 +4270,7 @@
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
@@ -4278,7 +4278,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -4288,7 +4288,7 @@
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
@@ -4296,7 +4296,7 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>62</v>
+        <v>45</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -4306,7 +4306,7 @@
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
@@ -4314,7 +4314,7 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -4324,7 +4324,7 @@
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
@@ -4332,7 +4332,7 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -4342,7 +4342,7 @@
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>258</v>
+        <v>249</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
@@ -4350,7 +4350,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -4360,15 +4360,15 @@
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>301</v>
+        <v>250</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>BLOCK C</t>
+          <t>BLOCK B</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -4378,15 +4378,15 @@
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>302</v>
+        <v>251</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>BLOCK C</t>
+          <t>BLOCK B</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -4396,15 +4396,15 @@
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>304</v>
+        <v>252</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>BLOCK C</t>
+          <t>BLOCK B</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>74</v>
+        <v>52</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -4414,15 +4414,15 @@
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>305</v>
+        <v>253</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>BLOCK C</t>
+          <t>BLOCK B</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>71</v>
+        <v>48</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -4432,15 +4432,15 @@
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>308</v>
+        <v>254</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>BLOCK C</t>
+          <t>BLOCK B</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>73</v>
+        <v>44</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -4450,15 +4450,15 @@
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>310</v>
+        <v>255</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>BLOCK C</t>
+          <t>BLOCK B</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>72</v>
+        <v>39</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -4468,15 +4468,15 @@
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>311</v>
+        <v>256</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>BLOCK C</t>
+          <t>BLOCK B</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>77</v>
+        <v>48</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -4486,15 +4486,15 @@
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>317</v>
+        <v>257</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>BLOCK C</t>
+          <t>BLOCK B</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -4504,15 +4504,15 @@
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>318</v>
+        <v>259</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>BLOCK C</t>
+          <t>BLOCK B</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -4522,15 +4522,15 @@
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>320</v>
+        <v>260</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>BLOCK C</t>
+          <t>BLOCK B</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -4540,7 +4540,7 @@
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>321</v>
+        <v>301</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
@@ -4548,7 +4548,7 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -4558,7 +4558,7 @@
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>323</v>
+        <v>306</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
@@ -4566,7 +4566,7 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>47</v>
+        <v>72</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
@@ -4576,7 +4576,7 @@
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>324</v>
+        <v>307</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
@@ -4594,7 +4594,7 @@
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>325</v>
+        <v>308</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
@@ -4602,7 +4602,7 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>49</v>
+        <v>70</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -4612,7 +4612,7 @@
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>326</v>
+        <v>309</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
@@ -4620,7 +4620,7 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>56</v>
+        <v>73</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -4630,7 +4630,7 @@
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>327</v>
+        <v>310</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
@@ -4638,7 +4638,7 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -4648,7 +4648,7 @@
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>331</v>
+        <v>311</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
@@ -4656,7 +4656,7 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
@@ -4666,7 +4666,7 @@
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>335</v>
+        <v>313</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
@@ -4674,7 +4674,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -4684,7 +4684,7 @@
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>337</v>
+        <v>314</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
@@ -4692,7 +4692,7 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -4702,7 +4702,7 @@
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>338</v>
+        <v>316</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
@@ -4710,7 +4710,7 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
@@ -4720,15 +4720,15 @@
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>401</v>
+        <v>317</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>BLOCK D</t>
+          <t>BLOCK C</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -4738,15 +4738,15 @@
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>405</v>
+        <v>318</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>BLOCK D</t>
+          <t>BLOCK C</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
@@ -4756,15 +4756,15 @@
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>406</v>
+        <v>319</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>BLOCK D</t>
+          <t>BLOCK C</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
@@ -4774,15 +4774,15 @@
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>407</v>
+        <v>320</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>BLOCK D</t>
+          <t>BLOCK C</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>64</v>
+        <v>44</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
@@ -4792,15 +4792,15 @@
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>408</v>
+        <v>322</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>BLOCK D</t>
+          <t>BLOCK C</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
@@ -4810,15 +4810,15 @@
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>410</v>
+        <v>323</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>BLOCK D</t>
+          <t>BLOCK C</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
@@ -4828,15 +4828,15 @@
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>413</v>
+        <v>324</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>BLOCK D</t>
+          <t>BLOCK C</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
@@ -4846,15 +4846,15 @@
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>417</v>
+        <v>325</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>BLOCK D</t>
+          <t>BLOCK C</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
@@ -4864,15 +4864,15 @@
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>418</v>
+        <v>326</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>BLOCK D</t>
+          <t>BLOCK C</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
@@ -4882,15 +4882,15 @@
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>419</v>
+        <v>328</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>BLOCK D</t>
+          <t>BLOCK C</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
@@ -4900,15 +4900,15 @@
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>421</v>
+        <v>329</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>BLOCK D</t>
+          <t>BLOCK C</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
@@ -4918,15 +4918,15 @@
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>424</v>
+        <v>330</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>BLOCK D</t>
+          <t>BLOCK C</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>61</v>
+        <v>81</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
@@ -4936,15 +4936,15 @@
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>425</v>
+        <v>331</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>BLOCK D</t>
+          <t>BLOCK C</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>54</v>
+        <v>78</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
@@ -4954,15 +4954,15 @@
     </row>
     <row r="112">
       <c r="A112" t="n">
-        <v>426</v>
+        <v>332</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>BLOCK D</t>
+          <t>BLOCK C</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>48</v>
+        <v>83</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
@@ -4972,15 +4972,15 @@
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>427</v>
+        <v>333</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>BLOCK D</t>
+          <t>BLOCK C</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>39</v>
+        <v>71</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
@@ -4990,15 +4990,15 @@
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>428</v>
+        <v>335</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>BLOCK D</t>
+          <t>BLOCK C</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>39</v>
+        <v>61</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
@@ -5008,15 +5008,15 @@
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>429</v>
+        <v>336</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>BLOCK D</t>
+          <t>BLOCK C</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
@@ -5026,15 +5026,15 @@
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>435</v>
+        <v>337</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>BLOCK D</t>
+          <t>BLOCK C</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
@@ -5044,15 +5044,15 @@
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>436</v>
+        <v>339</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>BLOCK D</t>
+          <t>BLOCK C</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
@@ -5062,7 +5062,7 @@
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>437</v>
+        <v>402</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
@@ -5070,7 +5070,7 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
@@ -5080,7 +5080,7 @@
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>439</v>
+        <v>403</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
@@ -5088,7 +5088,7 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
@@ -5098,7 +5098,7 @@
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>440</v>
+        <v>404</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
@@ -5106,7 +5106,7 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
@@ -5116,7 +5116,7 @@
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>441</v>
+        <v>405</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
@@ -5124,7 +5124,7 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
@@ -5134,7 +5134,7 @@
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>442</v>
+        <v>407</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
@@ -5142,7 +5142,7 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>51</v>
+        <v>64</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
@@ -5152,7 +5152,7 @@
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>444</v>
+        <v>409</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
@@ -5160,7 +5160,7 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
@@ -5170,7 +5170,7 @@
     </row>
     <row r="124">
       <c r="A124" t="n">
-        <v>446</v>
+        <v>412</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
@@ -5178,7 +5178,7 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
@@ -5188,7 +5188,7 @@
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>447</v>
+        <v>413</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
@@ -5196,7 +5196,7 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
@@ -5206,7 +5206,7 @@
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>448</v>
+        <v>414</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
@@ -5214,7 +5214,7 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
@@ -5224,17 +5224,395 @@
     </row>
     <row r="127">
       <c r="A127" t="n">
+        <v>415</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>BLOCK D</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>55</v>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Evaluator 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>416</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>BLOCK D</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>59</v>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Evaluator 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>418</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>BLOCK D</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>73</v>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Evaluator 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>419</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>BLOCK D</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>72</v>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Evaluator 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>421</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>BLOCK D</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>65</v>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Evaluator 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>422</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>BLOCK D</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>72</v>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Evaluator 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>423</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>BLOCK D</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>66</v>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Evaluator 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>424</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>BLOCK D</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>65</v>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Evaluator 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>425</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>BLOCK D</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>53</v>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Evaluator 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>427</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>BLOCK D</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>45</v>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Evaluator 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>428</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>BLOCK D</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>37</v>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Evaluator 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>430</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>BLOCK D</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>45</v>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Evaluator 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>432</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>BLOCK D</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>44</v>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Evaluator 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>436</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>BLOCK D</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>52</v>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Evaluator 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>437</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>BLOCK D</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>52</v>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Evaluator 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>438</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>BLOCK D</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>57</v>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Evaluator 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>440</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>BLOCK D</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>63</v>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Evaluator 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>443</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>BLOCK D</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>55</v>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Evaluator 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>446</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>BLOCK D</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>49</v>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Evaluator 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>447</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>BLOCK D</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>58</v>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Evaluator 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>449</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>BLOCK D</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>52</v>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Evaluator 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
         <v>450</v>
       </c>
-      <c r="B127" t="inlineStr">
+      <c r="B148" t="inlineStr">
         <is>
           <t>BLOCK D</t>
         </is>
       </c>
-      <c r="C127" t="n">
+      <c r="C148" t="n">
         <v>48</v>
       </c>
-      <c r="D127" t="inlineStr">
+      <c r="D148" t="inlineStr">
         <is>
           <t>Evaluator 1</t>
         </is>

</xml_diff>